<commit_message>
Add 死期 buff and ReduceBuff mechanics
Implement death-timer debuff and supporting plumbing: add new buff enums (死期, 黑无常, 白无常, 禁武令, 卸甲令, 监禁令) and many new card enums (ids 50-80). Introduce BuffEffects.ReduceBuff and an OnReduceBuff hook on IBuffEffectExecutor and IEntityController, plus ReduceBuff wrappers in EnemyController and PlayerController. Add new buff executor 死期 that counts down each turn and kills the entity when it reaches zero. Update existing buff executors with empty OnReduceBuff stubs. Update several card effect implementations (0013, 0014, 0015) to use card usage, apply damage/shield, handle kill/turn-end chances, and call ReduceBuff where appropriate. Append placeholder card entries and adjust mask/value arrays in cardtable.json. Add .meta for the new buff file and update source Excel config files. Overall this enables countdown-style debuffs and supports reducing buff parameters from card effects.
</commit_message>
<xml_diff>
--- a/Configs/source/Datas/__tables__.xlsx
+++ b/Configs/source/Datas/__tables__.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080"/>
+    <workbookView windowWidth="29100" windowHeight="12700"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
   <si>
     <t>##var</t>
   </si>
@@ -135,15 +135,6 @@
   </si>
   <si>
     <t>MaskTable@mask.xlsx</t>
-  </si>
-  <si>
-    <t>SpecialTable</t>
-  </si>
-  <si>
-    <t>SpecialConfig</t>
-  </si>
-  <si>
-    <t>SpecialTable@special.xlsx</t>
   </si>
 </sst>
 </file>
@@ -1089,12 +1080,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="2" max="2" width="20.375" customWidth="1"/>
     <col min="3" max="3" width="15.625" customWidth="1"/>
     <col min="4" max="4" width="32.375" customWidth="1"/>
-    <col min="5" max="5" width="43.6" customWidth="1"/>
+    <col min="5" max="5" width="43.5982142857143" customWidth="1"/>
     <col min="6" max="9" width="18" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1188,7 +1179,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="2:5">
       <c r="B4" t="s">
         <v>27</v>
       </c>
@@ -1202,7 +1193,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="2:5">
       <c r="B5" t="s">
         <v>30</v>
       </c>
@@ -1216,7 +1207,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="2:5">
       <c r="B6" t="s">
         <v>33</v>
       </c>
@@ -1230,30 +1221,19 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
-      <c r="B7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" t="b">
-        <v>1</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>38</v>
-      </c>
+    <row r="7" spans="5:5">
+      <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="5:5">
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="5:5">
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="5:5">
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="5:5">
       <c r="E11" s="2"/>
     </row>
   </sheetData>
@@ -1261,7 +1241,6 @@
     <hyperlink ref="E4" r:id="rId1" display="CardTable@card.xlsx" tooltip="mailto:CardTable@card.xlsx"/>
     <hyperlink ref="E5" r:id="rId2" display="GhostTable@ghost.xlsx"/>
     <hyperlink ref="E6" r:id="rId3" display="MaskTable@mask.xlsx"/>
-    <hyperlink ref="E7" r:id="rId4" display="SpecialTable@special.xlsx"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Add Mengpo configs and table; adjust card value
Add Mengpo data and runtime support: new resource mengpotable.json (mengpo_soup_effect entries), generated MengpoConfig and MengpoTable classes, and register/resolve MengpoTable in Tables. Also tweak a cardtable.json numeric value (5 -> 3) and update a comment in BuffEnum. Source Excel data (__tables__.xlsx and special.xlsx) were updated as well.
</commit_message>
<xml_diff>
--- a/Configs/source/Datas/__tables__.xlsx
+++ b/Configs/source/Datas/__tables__.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t>##var</t>
   </si>
@@ -135,6 +135,15 @@
   </si>
   <si>
     <t>MaskTable@mask.xlsx</t>
+  </si>
+  <si>
+    <t>MengpoTable</t>
+  </si>
+  <si>
+    <t>MengpoConfig</t>
+  </si>
+  <si>
+    <t>MengpoTable@special.xlsx</t>
   </si>
 </sst>
 </file>
@@ -1221,8 +1230,19 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="5:5">
-      <c r="E7" s="2"/>
+    <row r="7" spans="2:5">
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="8" spans="5:5">
       <c r="E8" s="2"/>
@@ -1241,6 +1261,7 @@
     <hyperlink ref="E4" r:id="rId1" display="CardTable@card.xlsx" tooltip="mailto:CardTable@card.xlsx"/>
     <hyperlink ref="E5" r:id="rId2" display="GhostTable@ghost.xlsx"/>
     <hyperlink ref="E6" r:id="rId3" display="MaskTable@mask.xlsx"/>
+    <hyperlink ref="E7" r:id="rId4" display="MengpoTable@special.xlsx"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>